<commit_message>
fix(ops): update all só pendentes WUD e endurecer Dozzle/AdGuard
O botão do HA passa a actualizar apenas containers com updateAvailable;
validação pré-update evita recreates sem users.yml/AdGuardHome.yaml.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Dispositivos - 2026.xlsx
+++ b/Dispositivos - 2026.xlsx
@@ -356,7 +356,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblClientes" displayName="tblClientes" ref="A1:I96" headerRowCount="1" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblClientes" displayName="tblClientes" ref="A1:I98" headerRowCount="1" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
   <autoFilter ref="A1:I99"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID do Cliente" dataDxfId="31">
@@ -929,13 +929,6 @@
         <v/>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
     <row r="16">
       <c r="C16" s="2" t="n"/>
     </row>
@@ -1128,12 +1121,6 @@
         <v/>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="C13" s="2" t="n"/>
     </row>
@@ -1832,7 +1819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I96"/>
+  <dimension ref="A1:I98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="20.44140625" customWidth="1" style="1" min="1" max="1"/>
@@ -2449,7 +2436,7 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="I15" s="4" t="n"/>
+      <c r="I15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -2489,7 +2476,7 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="I16" s="4" t="n"/>
+      <c r="I16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -2929,7 +2916,7 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="I27" s="4" t="n"/>
+      <c r="I27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
@@ -3289,7 +3276,7 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="I36" s="4" t="n"/>
+      <c r="I36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n">
@@ -5673,7 +5660,95 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="I96" s="4" t="n"/>
+      <c r="I96" s="7" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="7" t="n">
+        <v>99</v>
+      </c>
+      <c r="B97" s="9" t="inlineStr">
+        <is>
+          <t>Servidor</t>
+        </is>
+      </c>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>AdGuard Backup</t>
+        </is>
+      </c>
+      <c r="D97" s="7">
+        <f>IF(ISERROR(INDEX(tblGrupos[Rede],MATCH(tblClientes[[#This Row],[Plataforma]],tblGrupos[Plataforma],0))),"",INDEX(tblGrupos[Rede],MATCH(tblClientes[[#This Row],[Plataforma]],tblGrupos[Plataforma],0)))</f>
+        <v/>
+      </c>
+      <c r="E97" s="7" t="inlineStr">
+        <is>
+          <t>Servidor</t>
+        </is>
+      </c>
+      <c r="F97" s="7" t="inlineStr">
+        <is>
+          <t>192.168.3.22</t>
+        </is>
+      </c>
+      <c r="G97" s="7" t="inlineStr">
+        <is>
+          <t>Não se Aplica</t>
+        </is>
+      </c>
+      <c r="H97" s="9" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="I97" s="1" t="inlineStr">
+        <is>
+          <t>Pi Zero 2 W, MAC e4:5f:01:8f:21:d9. Wi-Fi Hangar com override UniFi para VLAN Servidor. DNS secundário.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>100</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Tuya</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Relógio Suíte</t>
+        </is>
+      </c>
+      <c r="D98">
+        <f>IF(ISERROR(INDEX(tblGrupos[Rede],MATCH(tblClientes[[#This Row],[Plataforma]],tblGrupos[Plataforma],0))),"",INDEX(tblGrupos[Rede],MATCH(tblClientes[[#This Row],[Plataforma]],tblGrupos[Plataforma],0)))</f>
+        <v/>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>IoT</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>192.168.2.59</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>MAC c0:f8:53:65:b9:77; Tuya eb3f4780d62224fe1epmtg; LocalTuya</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="3">

</xml_diff>